<commit_message>
Docs, deck and catalog for the friendlier responses: greeting, BOM, vendor comparison, order story, approval ladder, HTML update email
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Aj5vE1JNcAxiTqppU4PS2Y
</commit_message>
<xml_diff>
--- a/docs/LaunchKit_Provisioner_Agent_Catalog.xlsx
+++ b/docs/LaunchKit_Provisioner_Agent_Catalog.xlsx
@@ -517,7 +517,7 @@
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>The root agent acts as a front-line coordinator by taking the launch brief, registering the request and delegating to the brief analyst, sourcing planner and fulfilment agents in a fixed order. It shows the manager a decision card with three computed options and incorporates a critical human-in-the-loop sign-off gate: above the autopilot limit it starts an Application Integration approval, tells the user that an approval email was sent, and holds every order until the executive approves. Once approved it has the orders placed; if rejected it releases the held depot stock.</t>
+          <t>The root agent acts as a front-line coordinator by taking the launch brief, registering the request and delegating to the brief analyst, sourcing planner and fulfilment agents in a fixed order. It shows the manager a 3-choices table with three computed options and incorporates a critical human-in-the-loop sign-off gate: above the autopilot limit it starts an Application Integration approval, tells the user that an approval email was sent, and holds every order until the executive approves. Once approved it has the orders placed; if rejected it releases the held depot stock.</t>
         </is>
       </c>
       <c r="F1" s="3" t="inlineStr">
@@ -541,7 +541,7 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>The brief analyst agent turns the free-text brief into requirement lines in one call: creator kits personalised by hoodie size and power plug from the BigQuery creator list, showroom displays and sales folios spread over the regions.</t>
+          <t>The brief analyst agent turns the free-text brief into requirement lines in one call: guest welcome kits personalised by hoodie size and power plug from the BigQuery guest list, venue display stands and sales folders spread over the regions.</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -565,7 +565,7 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>The sourcing planner agent audits regional depot surplus and vendor lead times and computes three options (full new, smart depot rebalance, eco launch) with cost, delivery date, safety buffer before the in-hand deadline, savings and carbon. It re-plans when a vendor reports a delay.</t>
+          <t>The sourcing planner agent audits regional depot surplus and vendor lead times and computes three options (buy everything new, use our stock first, green option) with cost, delivery date, safety buffer before the in-hand deadline, savings and carbon. It re-plans when a vendor reports a delay.</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -679,7 +679,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>The root agent is the front-line coordinator. It takes the launch brief, registers the request and calls the three specialist agents in a fixed order: Brief Analyst, Sourcing Planner, then (after sign-off) Fulfilment. It shows the manager the decision card with three computed options and waits for a choice. It holds the human-in-the-loop sign-off gate: only the root can call authorize_launch. Spend within the autopilot limit is approved by policy; above it an Application Integration approval emails the VP (or the CMO for the largest tier) and nothing is ordered until they approve. When the user asks for the status it reads the decision and has the orders placed (Approved) or releases the held depot stock (Rejected). It writes every reply the user sees.</t>
+          <t>The root agent is the Event Procurement Assistant, the front-line coordinator. Underneath it is a purchase order, procurement and approval system, but it handles a whole event brief (many items, many vendors) instead of single items. On a greeting it shows what it can do and what it needs. It takes the event brief, registers the request and calls the three specialist agents in a fixed order: Brief Analyst, Sourcing Planner, then (after sign-off) Fulfilment. It shows the manager, in simple words with tables and icons, the shopping list (Bill of Materials), the vendor comparison and the 3-choices table and waits for a choice. It holds the human-in-the-loop sign-off gate: only the root can call authorize_launch. Spend within the autopilot limit is approved by policy; above it an Application Integration approval emails the VP (or the CMO for the largest tier) and nothing is ordered until they approve. When the user asks for the status it reads the decision and has the orders placed (Approved) or releases the held depot stock (Rejected). It writes every reply the user sees.</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr">
@@ -711,12 +711,12 @@
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>The brief analyst turns the free-text brief into requirement lines in one call: creator unboxing kits (hoodie size, power plug and engraving from the creator list), showroom counter displays and executive sales folios, spread over the regions. It reports the channel totals and the size and plug breakdown. It never invents a bundle type.</t>
+          <t>The brief analyst turns the free-text brief into requirement lines in one call: guest welcome kits (hoodie size, power plug and engraving from the guest list), venue display stands and executive sales folders, spread over the regions. It returns the shopping list (Bill of Materials): each bundle, each item, totals and where they go. It never invents a bundle type.</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>BigQuery: bundle_templates, creators, regional_split, requirement_lines, audit_log</t>
+          <t>BigQuery: bundle_templates, guests, regional_split, requirement_lines, audit_log</t>
         </is>
       </c>
     </row>
@@ -743,7 +743,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>The sourcing planner computes three options for the request from BigQuery data: full brand-new production, smart depot rebalance (reuses surplus stock from regional depots, nearest first, and picks vendors that keep the safety buffer) and a certified eco launch. Each option has cost, delivery date, buffer hours before the in-hand deadline, savings, carbon and risk. It re-plans when a vendor reports a delay. It never changes a number.</t>
+          <t>The sourcing planner computes three options for the request from BigQuery data: full brand-new production, use our stock first, buy the rest (reuses surplus stock from our warehouses, nearest first, and picks vendors that keep the safety buffer) and a certified green option. It also returns the vendor comparison (every vendor checked, who was chosen, why). Each option has cost, delivery date, buffer hours before the in-hand deadline, savings, carbon and risk. It re-plans when a vendor reports a delay. It never changes a number.</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
@@ -795,7 +795,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1105,32 +1105,32 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Brief Analyst Agent</t>
+          <t>Root Agent</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>build_requirements</t>
+          <t>show_capabilities</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Python tool (batch)</t>
+          <t>Python tool</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Expands every bundle of the brief into requirement lines per SKU and region; creator kits personalised from the creator list.</t>
+          <t>The hello card: what the assistant can do and what it needs from the user, with sample prompts.</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>bundle_templates, creators, regional_split, launch_requests</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>requirement_lines, audit_log</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
@@ -1140,39 +1140,39 @@
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>Unknown bundle type returns the valid types</t>
+          <t>Fixed text, no data access</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Sourcing Planner Agent</t>
+          <t>Root Agent</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>build_scenarios</t>
+          <t>get_approval_rules</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Python tool (batch)</t>
+          <t>Python tool</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>Computes and stores the three options with cost, delivery date, buffer, savings, carbon, risk; returns the decision card and whether autopilot applies.</t>
+          <t>The approval levels as a ladder (up to $5,000 automatic, up to $50,000 VP, above that CMO).</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>requirement_lines, vendor_offers, vendors, vendor_disruptions, v_depot_available, transit_lanes, assets, planning_rules, approval_policy</t>
+          <t>approval_policy</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>scenarios, scenario_lines, audit_log</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
@@ -1182,19 +1182,19 @@
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>Refuses to re-plan once a sign-off is pending or approved</t>
+          <t>Read only</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Sourcing Planner Agent</t>
+          <t>Root Agent</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>report_vendor_delay</t>
+          <t>get_vendor_report</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -1204,17 +1204,17 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Records a vendor delay (by id or name). Before a sign-off: re-plan. After: reports the impact on the buffer.</t>
+          <t>Vendor comparison for a request: every vendor checked per item, price, days to make, late vendors, who was chosen, stock we already own.</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>vendors, decisions, scenario_lines</t>
+          <t>requirement_lines, vendor_offers, vendor_disruptions, scenarios, scenario_lines, v_depot_available</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>vendor_disruptions, audit_log</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
@@ -1224,47 +1224,173 @@
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>Ambiguous vendor names are refused</t>
+          <t>Read only</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
+          <t>Brief Analyst Agent</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>build_requirements</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Python tool (batch)</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Expands every bundle of the brief into requirement lines per SKU and region; guest welcome kits personalised from the guest list. Returns the shopping list (Bill of Materials).</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>bundle_templates, guests, regional_split, launch_requests</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>requirement_lines, audit_log</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>Unknown bundle type returns the valid types</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Sourcing Planner Agent</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>build_scenarios</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Python tool (batch)</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Computes and stores the three options with cost, delivery date, buffer, savings, carbon, risk; returns the 3-choices table and whether autopilot applies.</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>requirement_lines, vendor_offers, vendors, vendor_disruptions, v_depot_available, transit_lanes, assets, planning_rules, approval_policy</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>scenarios, scenario_lines, audit_log</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>Refuses to re-plan once a sign-off is pending or approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Sourcing Planner Agent</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>report_vendor_delay</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>Python tool</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>Records a vendor delay (by id or name). Before a sign-off: re-plan. After: reports the impact on the buffer.</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>vendors, decisions, scenario_lines</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>vendor_disruptions, audit_log</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>Ambiguous vendor names are refused</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
           <t>Fulfilment Agent</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>execute_plan</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>Python tool (batch)</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>Places every line of the approved option: purchase orders, depot transfers (in parallel), then the tracking update; writes the results in bulk.</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E14" s="5" t="inlineStr">
         <is>
           <t>decisions, scenario_lines, launches, approvers</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="F14" s="5" t="inlineStr">
         <is>
           <t>purchase_orders, depot_transfers, scenario_lines (EXECUTED), depot_holds (CONSUMED), audit_log</t>
         </is>
       </c>
-      <c r="G11" s="6" t="inlineStr">
+      <c r="G14" s="5" t="inlineStr">
         <is>
           <t>create_purchase_order, create_depot_transfer, send_launch_update</t>
         </is>
       </c>
-      <c r="H11" s="6" t="inlineStr">
+      <c r="H14" s="5" t="inlineStr">
         <is>
           <t>BLOCKED unless APPROVED; never beyond the authorised amount; idempotent</t>
         </is>
@@ -1385,7 +1511,7 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>What goes into one creator kit, showroom display or sales folio.</t>
+          <t>What goes into one guest welcome kit, venue display stand or sales folder.</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
@@ -1402,7 +1528,7 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>creators</t>
+          <t>guests</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
@@ -1412,7 +1538,7 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>150 creators: hoodie size, region and power plug (personalisation).</t>
+          <t>150 guests: hoodie size, region and power plug (personalisation).</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
@@ -1439,7 +1565,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>How showroom and sales bundles spread over regions.</t>
+          <t>How venue and sales bundles spread over regions.</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -2292,7 +2418,7 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>Sends the brief in Gemini Enterprise: 150 creator kits, 10 showroom displays, 300 sales folios.</t>
+          <t>Sends the brief in Gemini Enterprise: 150 guest welcome kits, 10 venue display stands, 300 sales folders.</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
@@ -2357,7 +2483,7 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Reads bundle_templates, creators, regional_split; writes requirement_lines</t>
+          <t>Reads bundle_templates, guests, regional_split; writes requirement_lines</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -2412,7 +2538,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Shows the decision card and asks which option</t>
+          <t>Shows the 3-choices table and asks which option</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Docs: guided questions, single item, new events
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Aj5vE1JNcAxiTqppU4PS2Y
</commit_message>
<xml_diff>
--- a/docs/LaunchKit_Provisioner_Agent_Catalog.xlsx
+++ b/docs/LaunchKit_Provisioner_Agent_Catalog.xlsx
@@ -868,7 +868,7 @@
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>Validates the launch and creates the request (REQ-xxxx).</t>
+          <t>Finds the event by name or id (or creates a new event with the date given, or updates its date), validates the date, and creates the request (REQ-xxxx).</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
@@ -878,7 +878,7 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>launch_requests, audit_log</t>
+          <t>launches (new event or new date), launch_requests, audit_log</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
@@ -888,7 +888,7 @@
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>Unknown launch is refused</t>
+          <t>Unknown event without a date, or a date that is not in the future, is refused</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Docs: checklist, business advice, in-short box
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Aj5vE1JNcAxiTqppU4PS2Y
</commit_message>
<xml_diff>
--- a/docs/LaunchKit_Provisioner_Agent_Catalog.xlsx
+++ b/docs/LaunchKit_Provisioner_Agent_Catalog.xlsx
@@ -711,7 +711,7 @@
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>The brief analyst turns the free-text brief into requirement lines in one call: guest welcome kits (hoodie size, power plug and engraving from the guest list), venue display stands and executive sales folders, spread over the regions. It returns the shopping list (Bill of Materials): each bundle, each item, totals and where they go. It never invents a bundle type.</t>
+          <t>The brief analyst turns the free-text brief into requirement lines in one call: guest welcome kits (hoodie size, power plug and engraving from the guest list), venue display stands and executive sales folders, spread over the regions. It returns the shopping list (Bill of Materials) and business advice (spares, a kind of bundle left out, the rest of a bundle, a date that is too close). It never invents a bundle type.</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
@@ -795,7 +795,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1152,7 +1152,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>get_approval_rules</t>
+          <t>show_checklist</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -1162,12 +1162,12 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>The approval levels as a ladder (up to $5,000 automatic, up to $50,000 VP, above that CMO).</t>
+          <t>The three things to close on (event, date, what is needed) with ticks and the one next question, shown on every question turn.</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>approval_policy</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
@@ -1182,7 +1182,7 @@
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>Read only</t>
+          <t>Fixed wording, no data access</t>
         </is>
       </c>
     </row>
@@ -1194,7 +1194,7 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>get_vendor_report</t>
+          <t>get_approval_rules</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -1204,12 +1204,12 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Vendor comparison for a request: every vendor checked per item, price, days to make, late vendors, who was chosen, stock we already own.</t>
+          <t>The approval levels as a ladder (up to $5,000 automatic, up to $50,000 VP, above that CMO).</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>requirement_lines, vendor_offers, vendor_disruptions, scenarios, scenario_lines, v_depot_available</t>
+          <t>approval_policy</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
@@ -1231,32 +1231,32 @@
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Brief Analyst Agent</t>
+          <t>Root Agent</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>build_requirements</t>
+          <t>get_vendor_report</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Python tool (batch)</t>
+          <t>Python tool</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>Expands every bundle of the brief into requirement lines per SKU and region; guest welcome kits personalised from the guest list. Returns the shopping list (Bill of Materials).</t>
+          <t>Vendor comparison for a request: every vendor checked per item, price, days to make, late vendors, who was chosen, stock we already own.</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>bundle_templates, guests, regional_split, launch_requests</t>
+          <t>requirement_lines, vendor_offers, vendor_disruptions, scenarios, scenario_lines, v_depot_available</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>requirement_lines, audit_log</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
@@ -1266,19 +1266,19 @@
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>Unknown bundle type returns the valid types</t>
+          <t>Read only</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Sourcing Planner Agent</t>
+          <t>Brief Analyst Agent</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>build_scenarios</t>
+          <t>build_requirements</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -1288,17 +1288,17 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Computes and stores the three options with cost, delivery date, buffer, savings, carbon, risk; returns the 3-choices table and whether autopilot applies.</t>
+          <t>Expands every bundle of the brief into requirement lines per SKU and region; guest welcome kits personalised from the guest list. Returns the shopping list (Bill of Materials).</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>requirement_lines, vendor_offers, vendors, vendor_disruptions, v_depot_available, transit_lanes, assets, planning_rules, approval_policy</t>
+          <t>bundle_templates, guests, regional_split, launch_requests</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>scenarios, scenario_lines, audit_log</t>
+          <t>requirement_lines, audit_log</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>Refuses to re-plan once a sign-off is pending or approved</t>
+          <t>Unknown bundle type returns the valid types</t>
         </is>
       </c>
     </row>
@@ -1320,27 +1320,27 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>report_vendor_delay</t>
+          <t>build_scenarios</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Python tool</t>
+          <t>Python tool (batch)</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>Records a vendor delay (by id or name). Before a sign-off: re-plan. After: reports the impact on the buffer.</t>
+          <t>Computes and stores the three options with cost, delivery date, buffer, savings, carbon, risk; returns the 3-choices table and whether autopilot applies.</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>vendors, decisions, scenario_lines</t>
+          <t>requirement_lines, vendor_offers, vendors, vendor_disruptions, v_depot_available, transit_lanes, assets, planning_rules, approval_policy</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>vendor_disruptions, audit_log</t>
+          <t>scenarios, scenario_lines, audit_log</t>
         </is>
       </c>
       <c r="G13" s="6" t="inlineStr">
@@ -1350,47 +1350,89 @@
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>Ambiguous vendor names are refused</t>
+          <t>Refuses to re-plan once a sign-off is pending or approved</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
+          <t>Sourcing Planner Agent</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>report_vendor_delay</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Python tool</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Records a vendor delay (by id or name). Before a sign-off: re-plan. After: reports the impact on the buffer.</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>vendors, decisions, scenario_lines</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>vendor_disruptions, audit_log</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>Ambiguous vendor names are refused</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
           <t>Fulfilment Agent</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>execute_plan</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>Python tool (batch)</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>Places every line of the approved option: purchase orders, depot transfers (in parallel), then the tracking update; writes the results in bulk.</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E15" s="6" t="inlineStr">
         <is>
           <t>decisions, scenario_lines, launches, approvers</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="F15" s="6" t="inlineStr">
         <is>
           <t>purchase_orders, depot_transfers, scenario_lines (EXECUTED), depot_holds (CONSUMED), audit_log</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="G15" s="6" t="inlineStr">
         <is>
           <t>create_purchase_order, create_depot_transfer, send_launch_update</t>
         </is>
       </c>
-      <c r="H14" s="5" t="inlineStr">
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t>BLOCKED unless APPROVED; never beyond the authorised amount; idempotent</t>
         </is>

</xml_diff>

<commit_message>
Show what we can offer (packs and items with stock, best prices, ready-by dates) so the user picks instead of typing a list
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Aj5vE1JNcAxiTqppU4PS2Y
</commit_message>
<xml_diff>
--- a/docs/LaunchKit_Provisioner_Agent_Catalog.xlsx
+++ b/docs/LaunchKit_Provisioner_Agent_Catalog.xlsx
@@ -1162,12 +1162,12 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>The three things to close on (event, date, what is needed) with ticks and the one next question, shown on every question turn.</t>
+          <t>The four things to close on (whole campaign or selected items, campaign name, date, what they pick) with ticks and the one next question, shown on every question turn. When it is time to pick it also shows what we can offer: packs and single items with our stock, best vendor price, ready-by dates against the date and a faster option.</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>launches, assets, bundle_templates, vendor_offers, vendor_disruptions, v_depot_available</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
@@ -1182,7 +1182,7 @@
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>Fixed wording, no data access</t>
+          <t>Read only</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Richer catalog data (12 vendors, 19 items, extras with stock) and --refresh-reference to load it into an existing dataset
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Aj5vE1JNcAxiTqppU4PS2Y
</commit_message>
<xml_diff>
--- a/docs/LaunchKit_Provisioner_Agent_Catalog.xlsx
+++ b/docs/LaunchKit_Provisioner_Agent_Catalog.xlsx
@@ -1526,17 +1526,17 @@
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>Collateral catalog with ship factor (size / weight).</t>
+          <t>Item catalog (19 items) with ship factor (size / weight): pack items and campaign extras. Feeds the offer shown to the user.</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>Planner</t>
+          <t>Planner, offer, BOM</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>Setup script</t>
+          <t>Setup script; refresh with --refresh-reference</t>
         </is>
       </c>
     </row>
@@ -1769,17 +1769,17 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Price, lead time and carbon per vendor, SKU and variant (STANDARD / ECO).</t>
+          <t>Price, lead time and carbon per vendor, SKU and variant (STANDARD / ECO). 12 vendors, 51 offers, at least two vendors per item.</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Planner</t>
+          <t>Planner, offer, vendor report</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Setup script</t>
+          <t>Setup script; refresh with --refresh-reference</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Docs, demo script and catalog for the natural conversation (people and date, where we deliver, suggested plan, vendor prices by date, other dates)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Aj5vE1JNcAxiTqppU4PS2Y
</commit_message>
<xml_diff>
--- a/docs/LaunchKit_Provisioner_Agent_Catalog.xlsx
+++ b/docs/LaunchKit_Provisioner_Agent_Catalog.xlsx
@@ -1162,12 +1162,12 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>The four things to close on (whole campaign or selected items, campaign name, date, what they pick) with ticks and the one next question, shown on every question turn. When it is time to pick it also shows what we can offer: packs and single items with our stock, best vendor price, ready-by dates against the date and a faster option.</t>
+          <t>The interviewer: what we know so far (people, date, place, campaign name, picks) with ticks and the one next question, shown on every question turn. After the date it shows where we can deliver (USA, Canada, London, Singapore) with vendors and warehouses; after the place it shows what we can offer: packs and single items, our stock, the best vendor price for the date, ready-by dates, a faster option and a suggested plan for the headcount.</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>launches, assets, bundle_templates, vendor_offers, vendor_disruptions, v_depot_available</t>
+          <t>venues, vendors, assets, bundle_templates, vendor_offers, vendor_date_pricing, vendor_disruptions, v_depot_available</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
@@ -1449,7 +1449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1516,7 +1516,7 @@
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>assets</t>
+          <t>venues</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
@@ -1526,12 +1526,12 @@
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>Item catalog (19 items) with ship factor (size / weight): pack items and campaign extras. Feeds the offer shown to the user.</t>
+          <t>Where a campaign can be held (USA, Canada, London, Singapore) and the region that serves it.</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>Planner, offer, BOM</t>
+          <t>Interviewer (show_checklist)</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
@@ -1543,7 +1543,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>bundle_templates</t>
+          <t>vendor_date_pricing</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
@@ -1553,24 +1553,24 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>What goes into one guest welcome kit, venue display stand or sales folder.</t>
+          <t>Price factor by days ahead: early-bird discounts and rush charges, per vendor or for all vendors (*).</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Brief analyst</t>
+          <t>Planner, offer, dates table</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>Setup script</t>
+          <t>Setup script; refresh with --refresh-reference</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>guests</t>
+          <t>assets</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
@@ -1580,24 +1580,24 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>150 guests: hoodie size, region and power plug (personalisation).</t>
+          <t>Item catalog (19 items) with ship factor (size / weight): pack items and campaign extras. Feeds the offer shown to the user.</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Brief analyst</t>
+          <t>Planner, offer, BOM</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Setup script</t>
+          <t>Setup script; refresh with --refresh-reference</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>regional_split</t>
+          <t>bundle_templates</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -1607,7 +1607,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>How venue and sales bundles spread over regions.</t>
+          <t>What goes into one guest welcome kit, venue display stand or sales folder.</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -1624,7 +1624,7 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>depots</t>
+          <t>guests</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
@@ -1634,12 +1634,12 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Regional marketing depots (London, Dallas, Singapore).</t>
+          <t>150 guests: hoodie size, region and power plug (personalisation).</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>v_depot_available</t>
+          <t>Brief analyst</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
@@ -1651,7 +1651,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>depot_stock</t>
+          <t>regional_split</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
@@ -1661,12 +1661,12 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Surplus units on hand per depot and SKU.</t>
+          <t>How venue and sales bundles spread over regions.</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>v_depot_available</t>
+          <t>Brief analyst</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -1678,34 +1678,34 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
+          <t>depots</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Table</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Regional marketing depots (London, Dallas, Singapore).</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
           <t>v_depot_available</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>View</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>Free surplus = on hand minus active and consumed holds.</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>Planner, sign-off, overview</t>
-        </is>
-      </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Setup script</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>transit_lanes</t>
+          <t>depot_stock</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -1715,12 +1715,12 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Shipping days and cost between regions.</t>
+          <t>Surplus units on hand per depot and SKU.</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Planner</t>
+          <t>v_depot_available</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -1732,34 +1732,34 @@
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>vendors</t>
+          <t>v_depot_available</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Table</t>
+          <t>View</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Manufacturers and where they ship from.</t>
+          <t>Free surplus = on hand minus active and consumed holds.</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>Planner</t>
+          <t>Planner, sign-off, overview</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>Setup script</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>vendor_offers</t>
+          <t>transit_lanes</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
@@ -1769,24 +1769,24 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Price, lead time and carbon per vendor, SKU and variant (STANDARD / ECO). 12 vendors, 51 offers, at least two vendors per item.</t>
+          <t>Shipping days and cost between regions.</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Planner, offer, vendor report</t>
+          <t>Planner</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Setup script; refresh with --refresh-reference</t>
+          <t>Setup script</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>planning_rules</t>
+          <t>vendors</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
@@ -1796,7 +1796,7 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Minimum and target safety buffer, depot handling days, transfer carbon.</t>
+          <t>Manufacturers and where they ship from.</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
@@ -1806,14 +1806,14 @@
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>Setup script; editable</t>
+          <t>Setup script</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>approval_policy</t>
+          <t>vendor_offers</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
@@ -1823,24 +1823,24 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Tiers: AUTOPILOT up to $5,000, VP sign-off up to $50,000, CMO above.</t>
+          <t>Price, lead time and carbon per vendor, SKU and variant (STANDARD / ECO). 12 vendors, 51 offers, at least two vendors per item.</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Sign-off</t>
+          <t>Planner, offer, vendor report</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Setup script; editable</t>
+          <t>Setup script; refresh with --refresh-reference</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>approvers</t>
+          <t>planning_rules</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
@@ -1850,24 +1850,24 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Emails per role (VP Product Marketing, CMO, Launch Team).</t>
+          <t>Minimum and target safety buffer, depot handling days, transfer carbon.</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>Sign-off, fulfilment</t>
+          <t>Planner</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>Setup script (--approver-email)</t>
+          <t>Setup script; editable</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>launch_requests</t>
+          <t>approval_policy</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
@@ -1877,24 +1877,24 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Every brief registered by the root agent.</t>
+          <t>Tiers: AUTOPILOT up to $5,000, VP sign-off up to $50,000, CMO above.</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Root</t>
+          <t>Sign-off</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Root</t>
+          <t>Setup script; editable</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>requirement_lines</t>
+          <t>approvers</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
@@ -1904,24 +1904,24 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>The brief broken down per SKU and destination region.</t>
+          <t>Emails per role (VP Product Marketing, CMO, Launch Team).</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>Planner</t>
+          <t>Sign-off, fulfilment</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>Brief analyst</t>
+          <t>Setup script (--approver-email)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>scenarios</t>
+          <t>launch_requests</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
@@ -1931,24 +1931,24 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>The computed options per request (cost, delivery, buffer, carbon, risk, recommended).</t>
+          <t>Every brief registered by the root agent.</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Root, sign-off</t>
+          <t>Root</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Sourcing planner</t>
+          <t>Root</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>scenario_lines</t>
+          <t>requirement_lines</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
@@ -1958,24 +1958,24 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>What each option does per line: reuse a depot or buy from a vendor; execution status.</t>
+          <t>The brief broken down per SKU and destination region.</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Sign-off, fulfilment</t>
+          <t>Planner</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>Sourcing planner, fulfilment</t>
+          <t>Brief analyst</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>decisions</t>
+          <t>scenarios</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
@@ -1985,24 +1985,24 @@
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>The sign-off on the chosen option: tier, approver, status, workflow execution id.</t>
+          <t>The computed options per request (cost, delivery, buffer, carbon, risk, recommended).</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Root, fulfilment</t>
+          <t>Root, sign-off</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>Root (authorize_launch, get_launch_status)</t>
+          <t>Sourcing planner</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>depot_holds</t>
+          <t>scenario_lines</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
@@ -2012,24 +2012,24 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Surplus stock held for a pending or approved option (ACTIVE / CONSUMED / RELEASED).</t>
+          <t>What each option does per line: reuse a depot or buy from a vendor; execution status.</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>v_depot_available</t>
+          <t>Sign-off, fulfilment</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>Root, fulfilment</t>
+          <t>Sourcing planner, fulfilment</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>vendor_disruptions</t>
+          <t>decisions</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
@@ -2039,24 +2039,24 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Reported vendor delays added to lead times.</t>
+          <t>The sign-off on the chosen option: tier, approver, status, workflow execution id.</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Planner</t>
+          <t>Root, fulfilment</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>Sourcing planner</t>
+          <t>Root (authorize_launch, get_launch_status)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>purchase_orders</t>
+          <t>depot_holds</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
@@ -2066,24 +2066,24 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Purchase orders issued through Application Integration.</t>
+          <t>Surplus stock held for a pending or approved option (ACTIVE / CONSUMED / RELEASED).</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
+          <t>v_depot_available</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
           <t>Root, fulfilment</t>
-        </is>
-      </c>
-      <c r="E23" s="6" t="inlineStr">
-        <is>
-          <t>Fulfilment</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>depot_transfers</t>
+          <t>vendor_disruptions</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -2093,69 +2093,123 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Depot-to-region stock transfers.</t>
+          <t>Reported vendor delays added to lead times.</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Root, fulfilment</t>
+          <t>Planner</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>Fulfilment</t>
+          <t>Sourcing planner</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>v_launch_readiness</t>
+          <t>purchase_orders</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>View</t>
+          <t>Table</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>Per request: chosen option, sign-off status, buffer, readiness colour, lines executed.</t>
+          <t>Purchase orders issued through Application Integration.</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>Overview</t>
+          <t>Root, fulfilment</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Fulfilment</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
+          <t>depot_transfers</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Table</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Depot-to-region stock transfers.</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Root, fulfilment</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Fulfilment</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>v_launch_readiness</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>Per request: chosen option, sign-off status, buffer, readiness colour, lines executed.</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
           <t>audit_log</t>
         </is>
       </c>
-      <c r="B26" s="5" t="inlineStr">
+      <c r="B28" s="5" t="inlineStr">
         <is>
           <t>Table</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr">
+      <c r="C28" s="5" t="inlineStr">
         <is>
           <t>Every governed action: who, what, when.</t>
         </is>
       </c>
-      <c r="D26" s="5" t="inlineStr">
+      <c r="D28" s="5" t="inlineStr">
         <is>
           <t>Root (get_audit_trail)</t>
         </is>
       </c>
-      <c r="E26" s="5" t="inlineStr">
+      <c r="E28" s="5" t="inlineStr">
         <is>
           <t>All agents and flows</t>
         </is>

</xml_diff>

<commit_message>
Campaign name ideas, and the campaign is created as soon as it is named
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Aj5vE1JNcAxiTqppU4PS2Y
</commit_message>
<xml_diff>
--- a/docs/LaunchKit_Provisioner_Agent_Catalog.xlsx
+++ b/docs/LaunchKit_Provisioner_Agent_Catalog.xlsx
@@ -795,7 +795,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1194,7 +1194,7 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>get_approval_rules</t>
+          <t>create_campaign</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -1204,17 +1204,17 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>The approval levels as a ladder (up to $5,000 automatic, up to $50,000 VP, above that CMO).</t>
+          <t>Creates the campaign as soon as the user has picked one of the name ideas or typed their own (or finds it if it exists) and shows a confirmation card.</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>approval_policy</t>
+          <t>launches</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>launches, audit_log</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>Read only</t>
+          <t>Needs a future date; never duplicates a campaign</t>
         </is>
       </c>
     </row>
@@ -1236,7 +1236,7 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>get_vendor_report</t>
+          <t>get_approval_rules</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -1246,12 +1246,12 @@
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>Vendor comparison for a request: every vendor checked per item, price, days to make, late vendors, who was chosen, stock we already own.</t>
+          <t>The approval levels as a ladder (up to $5,000 automatic, up to $50,000 VP, above that CMO).</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>requirement_lines, vendor_offers, vendor_disruptions, scenarios, scenario_lines, v_depot_available</t>
+          <t>approval_policy</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
@@ -1273,32 +1273,32 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Brief Analyst Agent</t>
+          <t>Root Agent</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>build_requirements</t>
+          <t>get_vendor_report</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Python tool (batch)</t>
+          <t>Python tool</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Expands every bundle of the brief into requirement lines per SKU and region; guest welcome kits personalised from the guest list. Returns the shopping list (Bill of Materials).</t>
+          <t>Vendor comparison for a request: every vendor checked per item, price, days to make, late vendors, who was chosen, stock we already own.</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>bundle_templates, guests, regional_split, launch_requests</t>
+          <t>requirement_lines, vendor_offers, vendor_disruptions, scenarios, scenario_lines, v_depot_available</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>requirement_lines, audit_log</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
@@ -1308,19 +1308,19 @@
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>Unknown bundle type returns the valid types</t>
+          <t>Read only</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>Sourcing Planner Agent</t>
+          <t>Brief Analyst Agent</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>build_scenarios</t>
+          <t>build_requirements</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
@@ -1330,17 +1330,17 @@
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>Computes and stores the three options with cost, delivery date, buffer, savings, carbon, risk; returns the 3-choices table and whether autopilot applies.</t>
+          <t>Expands every bundle of the brief into requirement lines per SKU and region; guest welcome kits personalised from the guest list. Returns the shopping list (Bill of Materials).</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>requirement_lines, vendor_offers, vendors, vendor_disruptions, v_depot_available, transit_lanes, assets, planning_rules, approval_policy</t>
+          <t>bundle_templates, guests, regional_split, launch_requests</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>scenarios, scenario_lines, audit_log</t>
+          <t>requirement_lines, audit_log</t>
         </is>
       </c>
       <c r="G13" s="6" t="inlineStr">
@@ -1350,7 +1350,7 @@
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>Refuses to re-plan once a sign-off is pending or approved</t>
+          <t>Unknown bundle type returns the valid types</t>
         </is>
       </c>
     </row>
@@ -1362,27 +1362,27 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>report_vendor_delay</t>
+          <t>build_scenarios</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Python tool</t>
+          <t>Python tool (batch)</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Records a vendor delay (by id or name). Before a sign-off: re-plan. After: reports the impact on the buffer.</t>
+          <t>Computes and stores the three options with cost, delivery date, buffer, savings, carbon, risk; returns the 3-choices table and whether autopilot applies.</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>vendors, decisions, scenario_lines</t>
+          <t>requirement_lines, vendor_offers, vendors, vendor_disruptions, v_depot_available, transit_lanes, assets, planning_rules, approval_policy</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>vendor_disruptions, audit_log</t>
+          <t>scenarios, scenario_lines, audit_log</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -1392,47 +1392,89 @@
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>Ambiguous vendor names are refused</t>
+          <t>Refuses to re-plan once a sign-off is pending or approved</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
+          <t>Sourcing Planner Agent</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>report_vendor_delay</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>Python tool</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>Records a vendor delay (by id or name). Before a sign-off: re-plan. After: reports the impact on the buffer.</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>vendors, decisions, scenario_lines</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>vendor_disruptions, audit_log</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>Ambiguous vendor names are refused</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
           <t>Fulfilment Agent</t>
         </is>
       </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>execute_plan</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>Python tool (batch)</t>
         </is>
       </c>
-      <c r="D15" s="6" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>Places every line of the approved option: purchase orders, depot transfers (in parallel), then the tracking update; writes the results in bulk.</t>
         </is>
       </c>
-      <c r="E15" s="6" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>decisions, scenario_lines, launches, approvers</t>
         </is>
       </c>
-      <c r="F15" s="6" t="inlineStr">
+      <c r="F16" s="5" t="inlineStr">
         <is>
           <t>purchase_orders, depot_transfers, scenario_lines (EXECUTED), depot_holds (CONSUMED), audit_log</t>
         </is>
       </c>
-      <c r="G15" s="6" t="inlineStr">
+      <c r="G16" s="5" t="inlineStr">
         <is>
           <t>create_purchase_order, create_depot_transfer, send_launch_update</t>
         </is>
       </c>
-      <c r="H15" s="6" t="inlineStr">
+      <c r="H16" s="5" t="inlineStr">
         <is>
           <t>BLOCKED unless APPROVED; never beyond the authorised amount; idempotent</t>
         </is>

</xml_diff>

<commit_message>
HTML approval email with Approve and Reject buttons, shopping list and vendor table; orders-placed email gets shopping list, vendors and PO numbers; the approval task no longer sends Google's plain email
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Aj5vE1JNcAxiTqppU4PS2Y
</commit_message>
<xml_diff>
--- a/docs/LaunchKit_Provisioner_Agent_Catalog.xlsx
+++ b/docs/LaunchKit_Provisioner_Agent_Catalog.xlsx
@@ -2336,7 +2336,7 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>Create a purchase order for a vendor line of the approved option.</t>
+          <t>Create one purchase order per vendor for the approved option (all of that vendor's items together).</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
@@ -2378,7 +2378,7 @@
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>Create a stock transfer from a depot to a destination region.</t>
+          <t>Create one stock transfer per warehouse for the approved option (all items together).</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">

</xml_diff>